<commit_message>
chore: update sample kenya.xlsx report
</commit_message>
<xml_diff>
--- a/reports/kenya.xlsx
+++ b/reports/kenya.xlsx
@@ -17,48 +17,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="91">
   <si>
     <t>Sovereign Distress Assessment: Kenya</t>
   </si>
   <si>
-    <t>As-of Date: 2024-06-30 00:00:00 | Scenario: base | Simulation Draws: 100,000</t>
+    <t>As-of Date: 2024-09-30 00:00:00 | Scenario: base | Simulation Draws: 100,000</t>
   </si>
   <si>
     <t>12M DISTRESS PROBABILITY</t>
   </si>
   <si>
-    <t>97.8%</t>
+    <t>97.2%</t>
   </si>
   <si>
     <t>24M DISTRESS PROBABILITY</t>
   </si>
   <si>
-    <t>98.2%</t>
+    <t>97.6%</t>
   </si>
   <si>
     <t>EXPECTED NPV HAIRCUT</t>
   </si>
   <si>
-    <t>39.2%</t>
+    <t>38.4%</t>
   </si>
   <si>
     <t>12M EXPECTED LOSS</t>
   </si>
   <si>
-    <t>38.3%</t>
+    <t>37.3%</t>
   </si>
   <si>
     <t>FAIR VALUE BOND PRICE</t>
   </si>
   <si>
-    <t>61.7</t>
+    <t>62.7</t>
   </si>
   <si>
     <t>MEDIAN DURATION</t>
   </si>
   <si>
-    <t>30.1 mos</t>
+    <t>29.9 mos</t>
   </si>
   <si>
     <t>Headline Risk &amp; Valuation Metrics</t>
@@ -88,12 +88,6 @@
     <t>Median Resolution Duration (months)</t>
   </si>
   <si>
-    <t>Market Bond Price</t>
-  </si>
-  <si>
-    <t>Market Price Gap (Market - Model)</t>
-  </si>
-  <si>
     <t>Scenario Stress Testing Comparison</t>
   </si>
   <si>
@@ -274,10 +268,10 @@
     <t>external_debt_pct_gdp</t>
   </si>
   <si>
+    <t>imf_off_track_interaction</t>
+  </si>
+  <si>
     <t>imf_program</t>
-  </si>
-  <si>
-    <t>fiscal_balance_pct_gdp</t>
   </si>
   <si>
     <t>Fundamental Model vs Market Pricing</t>
@@ -563,22 +557,19 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Summary'!$A$17:$A$22</c:f>
+              <c:f>'Executive Summary'!$A$17:$A$20</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Scenario</c:v>
+                </c:pt>
                 <c:pt idx="1">
-                  <c:v>Scenario Stress Testing Comparison</c:v>
+                  <c:v>base</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Scenario</c:v>
+                  <c:v>fx_shock</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>base</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>fx_shock</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>spread_widening</c:v>
                 </c:pt>
               </c:strCache>
@@ -586,21 +577,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Summary'!$B$17:$B$22</c:f>
+              <c:f>'Executive Summary'!$B$17:$B$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.972</c:v>
+                </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.9904999999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.978</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.987</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.9865999999999999</c:v>
+                  <c:v>0.9834000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -624,22 +615,19 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Summary'!$A$17:$A$22</c:f>
+              <c:f>'Executive Summary'!$A$17:$A$20</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Scenario</c:v>
+                </c:pt>
                 <c:pt idx="1">
-                  <c:v>Scenario Stress Testing Comparison</c:v>
+                  <c:v>base</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Scenario</c:v>
+                  <c:v>fx_shock</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>base</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>fx_shock</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>spread_widening</c:v>
                 </c:pt>
               </c:strCache>
@@ -647,21 +635,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Summary'!$C$17:$C$22</c:f>
+              <c:f>'Executive Summary'!$C$17:$C$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.9761</c:v>
+                </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.99</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.9818000000000001</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.9881</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.9883</c:v>
+                  <c:v>0.9849</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -685,22 +673,19 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Summary'!$A$17:$A$22</c:f>
+              <c:f>'Executive Summary'!$A$17:$A$20</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Scenario</c:v>
+                </c:pt>
                 <c:pt idx="1">
-                  <c:v>Scenario Stress Testing Comparison</c:v>
+                  <c:v>base</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Scenario</c:v>
+                  <c:v>fx_shock</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>base</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>fx_shock</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>spread_widening</c:v>
                 </c:pt>
               </c:strCache>
@@ -708,21 +693,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Summary'!$E$17:$E$22</c:f>
+              <c:f>'Executive Summary'!$E$17:$E$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.373</c:v>
+                </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.3802</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.383</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.3865</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.3863</c:v>
+                  <c:v>0.3774</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1076,25 +1061,25 @@
                   <c:v>0.08</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.196</c:v>
+                  <c:v>0.1972</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.30035</c:v>
+                  <c:v>0.30205</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4047</c:v>
+                  <c:v>0.4069</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.491</c:v>
+                  <c:v>0.4933999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5773</c:v>
+                  <c:v>0.5799</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.7216250000000001</c:v>
+                  <c:v>0.7248749999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.80822</c:v>
+                  <c:v>0.8118599999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1159,25 +1144,25 @@
                   <c:v>0.92</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.804</c:v>
+                  <c:v>0.8028</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.69965</c:v>
+                  <c:v>0.6979500000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5952999999999999</c:v>
+                  <c:v>0.5931</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.509</c:v>
+                  <c:v>0.5066000000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.4227</c:v>
+                  <c:v>0.4201</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2783749999999999</c:v>
+                  <c:v>0.2751250000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.19178</c:v>
+                  <c:v>0.1881400000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1320,10 +1305,10 @@
                   <c:v>external_debt_pct_gdp</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>imf_off_track_interaction</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>imf_program</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>fiscal_balance_pct_gdp</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1335,22 +1320,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>5.465261556333266</c:v>
+                  <c:v>5.401214534677748</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1.295</c:v>
+                  <c:v>-1.435</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.278</c:v>
+                  <c:v>1.2555</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.275</c:v>
+                  <c:v>1.146</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>-0.65</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.312</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1864,7 +1849,7 @@
   <sheetPr>
     <tabColor rgb="FF1B365D"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1942,10 +1927,10 @@
         <v>18</v>
       </c>
       <c r="B9" s="8">
-        <v>0.978</v>
+        <v>0.972</v>
       </c>
       <c r="C9" s="8">
-        <v>0.9818000000000001</v>
+        <v>0.9761</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1953,10 +1938,10 @@
         <v>19</v>
       </c>
       <c r="B10" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3838</v>
       </c>
       <c r="C10" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3838</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1964,10 +1949,10 @@
         <v>20</v>
       </c>
       <c r="B11" s="8">
-        <v>0.383</v>
+        <v>0.373</v>
       </c>
       <c r="C11" s="8">
-        <v>0.3845</v>
+        <v>0.3746</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1975,10 +1960,10 @@
         <v>21</v>
       </c>
       <c r="B12" s="9">
-        <v>61.7</v>
+        <v>62.7</v>
       </c>
       <c r="C12" s="9">
-        <v>61.55</v>
+        <v>62.54</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1986,57 +1971,75 @@
         <v>22</v>
       </c>
       <c r="B13" s="9">
-        <v>30.1</v>
+        <v>29.9</v>
       </c>
       <c r="C13" s="9">
-        <v>30.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="7" t="s">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="9">
-        <v>82.5</v>
-      </c>
-      <c r="C14" s="9">
-        <v>82.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="7" t="s">
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="9">
-        <v>20.8</v>
-      </c>
-      <c r="C15" s="9">
-        <v>20.8</v>
+      <c r="B17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
-        <v>25</v>
+      <c r="A18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="8">
+        <v>0.972</v>
+      </c>
+      <c r="C18" s="8">
+        <v>0.9761</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0.3838</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0.373</v>
+      </c>
+      <c r="F18" s="9">
+        <v>62.7</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>31</v>
+      </c>
+      <c r="B19" s="8">
+        <v>0.9904999999999999</v>
+      </c>
+      <c r="C19" s="8">
+        <v>0.99</v>
+      </c>
+      <c r="D19" s="8">
+        <v>0.3838</v>
+      </c>
+      <c r="E19" s="8">
+        <v>0.3802</v>
+      </c>
+      <c r="F19" s="9">
+        <v>61.98</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2044,19 +2047,19 @@
         <v>32</v>
       </c>
       <c r="B20" s="8">
-        <v>0.978</v>
+        <v>0.9834000000000001</v>
       </c>
       <c r="C20" s="8">
-        <v>0.9818000000000001</v>
+        <v>0.9849</v>
       </c>
       <c r="D20" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3838</v>
       </c>
       <c r="E20" s="8">
-        <v>0.383</v>
+        <v>0.3774</v>
       </c>
       <c r="F20" s="9">
-        <v>61.7</v>
+        <v>62.26</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2064,59 +2067,19 @@
         <v>33</v>
       </c>
       <c r="B21" s="8">
-        <v>0.987</v>
+        <v>0.9626</v>
       </c>
       <c r="C21" s="8">
-        <v>0.9881</v>
+        <v>0.968</v>
       </c>
       <c r="D21" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3957</v>
       </c>
       <c r="E21" s="8">
-        <v>0.3865</v>
+        <v>0.3809</v>
       </c>
       <c r="F21" s="9">
-        <v>61.35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="8">
-        <v>0.9865999999999999</v>
-      </c>
-      <c r="C22" s="8">
-        <v>0.9883</v>
-      </c>
-      <c r="D22" s="8">
-        <v>0.3915999999999999</v>
-      </c>
-      <c r="E22" s="8">
-        <v>0.3863</v>
-      </c>
-      <c r="F22" s="9">
-        <v>61.37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="8">
-        <v>0.9884000000000001</v>
-      </c>
-      <c r="C23" s="8">
-        <v>0.9893999999999999</v>
-      </c>
-      <c r="D23" s="8">
-        <v>0.4036</v>
-      </c>
-      <c r="E23" s="8">
-        <v>0.3989</v>
-      </c>
-      <c r="F23" s="9">
-        <v>60.11</v>
+        <v>61.91</v>
       </c>
     </row>
   </sheetData>
@@ -2140,62 +2103,62 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" s="8">
-        <v>0.067</v>
+        <v>0.066</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3838</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B8" s="8">
-        <v>0.3915999999999999</v>
+        <v>0.3838</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B9" s="8">
-        <v>0.52866</v>
+        <v>0.5181300000000001</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10" s="8">
         <v>0.2</v>
@@ -2203,7 +2166,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B11" s="8">
         <v>0.6</v>
@@ -2211,20 +2174,20 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B15" s="8">
         <v>0.04</v>
@@ -2232,7 +2195,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B16" s="8">
         <v>0.12</v>
@@ -2240,7 +2203,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B17" s="8">
         <v>0.28</v>
@@ -2248,7 +2211,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B18" s="8">
         <v>0.32</v>
@@ -2256,7 +2219,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B19" s="8">
         <v>0.15</v>
@@ -2264,7 +2227,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B20" s="8">
         <v>0.06</v>
@@ -2272,7 +2235,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B21" s="8">
         <v>0.02</v>
@@ -2280,7 +2243,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B22" s="8">
         <v>0.01</v>
@@ -2306,33 +2269,33 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B6" s="8">
         <v>0.08</v>
@@ -2343,79 +2306,79 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B7" s="8">
-        <v>0.196</v>
+        <v>0.1972</v>
       </c>
       <c r="C7" s="8">
-        <v>0.804</v>
+        <v>0.8028</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B8" s="8">
-        <v>0.30035</v>
+        <v>0.30205</v>
       </c>
       <c r="C8" s="8">
-        <v>0.69965</v>
+        <v>0.6979500000000001</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B9" s="8">
-        <v>0.4047</v>
+        <v>0.4069</v>
       </c>
       <c r="C9" s="8">
-        <v>0.5952999999999999</v>
+        <v>0.5931</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B10" s="8">
-        <v>0.491</v>
+        <v>0.4933999999999999</v>
       </c>
       <c r="C10" s="8">
-        <v>0.509</v>
+        <v>0.5066000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="8">
-        <v>0.5773</v>
+        <v>0.5799</v>
       </c>
       <c r="C11" s="8">
-        <v>0.4227</v>
+        <v>0.4201</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B12" s="8">
-        <v>0.7216250000000001</v>
+        <v>0.7248749999999999</v>
       </c>
       <c r="C12" s="8">
-        <v>0.2783749999999999</v>
+        <v>0.2751250000000001</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B13" s="8">
-        <v>0.80822</v>
+        <v>0.8118599999999999</v>
       </c>
       <c r="C13" s="8">
-        <v>0.19178</v>
+        <v>0.1881400000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2438,120 +2401,120 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B6" s="9">
-        <v>6.429719478039138</v>
+        <v>6.354370040797351</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D6" s="9">
-        <v>5.465261556333266</v>
+        <v>5.401214534677748</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B7" s="9">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D7" s="9">
-        <v>-1.295</v>
+        <v>-1.435</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="9">
-        <v>28.4</v>
+        <v>27.9</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D8" s="9">
-        <v>1.278</v>
+        <v>1.2555</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="9">
-        <v>42.5</v>
+        <v>38.2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D9" s="9">
-        <v>1.275</v>
+        <v>1.146</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10" s="9">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D10" s="9">
-        <v>-0.65</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11" s="9">
-        <v>-5.2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>80</v>
       </c>
       <c r="D11" s="9">
-        <v>0.312</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2559,27 +2522,27 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B17" s="8">
-        <v>0.978</v>
+        <v>0.972</v>
       </c>
       <c r="C17" s="8">
-        <v>0.09817368539704707</v>
+        <v>0.09138456064369226</v>
       </c>
       <c r="D17" s="8">
-        <v>0.8798263146029529</v>
+        <v>0.8806154393563078</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2587,24 +2550,24 @@
         <v>20</v>
       </c>
       <c r="B18" s="8">
-        <v>0.383</v>
+        <v>0.373</v>
       </c>
       <c r="C18" s="8">
-        <v>0.05890421123822825</v>
+        <v>0.05483073638621536</v>
       </c>
       <c r="D18" s="8">
-        <v>0.3240957887617717</v>
+        <v>0.3181692636137846</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B19" s="9">
-        <v>620</v>
+        <v>575</v>
       </c>
       <c r="C19" s="9">
-        <v>620</v>
+        <v>575</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>

</xml_diff>